<commit_message>
Add optional OCC/external job links to vacancy template and cards.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/assets/bolsa/plantilla-vacantes-yaavs.xlsx
+++ b/assets/bolsa/plantilla-vacantes-yaavs.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vacantes'!$A$1:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vacantes'!$A$1:$I$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +33,13 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00003087"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -43,20 +49,14 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00003087"/>
-      <sz val="12"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="0064748B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
+      <b val="1"/>
       <color rgb="00003087"/>
-      <sz val="10"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="7">
@@ -73,11 +73,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F4FC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF8E1"/>
       </patternFill>
     </fill>
@@ -89,6 +84,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4FC"/>
       </patternFill>
     </fill>
   </fills>
@@ -118,30 +118,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -262,6 +261,11 @@
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>Sí = vacante abierta en web · No = solo catálogo</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Pega el link de OCC, Computrabajo, Indeed, LinkedIn, etc. Si está vacío, no se muestra botón externo.</t>
       </text>
     </comment>
   </commentList>
@@ -557,20 +561,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="58" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="40" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Puesto</t>
@@ -611,11 +616,16 @@
           <t>¿Abierta?</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Link OCC / externo (opcional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Solo llena estas columnas. Una fila = una vacante. Lo demás no se publica en la web.</t>
+          <t>Solo llena estas columnas. Una fila = una vacante. El link OCC/externo es opcional: si lo pegas, aparece un botón «Ver en OCC» (o similar) en la web.</t>
         </is>
       </c>
     </row>
@@ -660,6 +670,11 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.occ.com.mx/empleo/oferta/ejemplo-asesor-att</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -702,6 +717,7 @@
           <t>Sí</t>
         </is>
       </c>
+      <c r="I4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -744,6 +760,7 @@
           <t>No</t>
         </is>
       </c>
+      <c r="I5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="6" t="inlineStr"/>
@@ -754,6 +771,7 @@
       <c r="F6" s="6" t="inlineStr"/>
       <c r="G6" s="6" t="inlineStr"/>
       <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="6" t="inlineStr"/>
@@ -764,6 +782,7 @@
       <c r="F7" s="6" t="inlineStr"/>
       <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="6" t="inlineStr"/>
@@ -774,6 +793,7 @@
       <c r="F8" s="6" t="inlineStr"/>
       <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="6" t="inlineStr"/>
@@ -784,6 +804,7 @@
       <c r="F9" s="6" t="inlineStr"/>
       <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="6" t="inlineStr"/>
@@ -794,6 +815,7 @@
       <c r="F10" s="6" t="inlineStr"/>
       <c r="G10" s="6" t="inlineStr"/>
       <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="6" t="inlineStr"/>
@@ -804,6 +826,7 @@
       <c r="F11" s="6" t="inlineStr"/>
       <c r="G11" s="6" t="inlineStr"/>
       <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="6" t="inlineStr"/>
@@ -814,6 +837,7 @@
       <c r="F12" s="6" t="inlineStr"/>
       <c r="G12" s="6" t="inlineStr"/>
       <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="6" t="inlineStr"/>
@@ -824,6 +848,7 @@
       <c r="F13" s="6" t="inlineStr"/>
       <c r="G13" s="6" t="inlineStr"/>
       <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="6" t="inlineStr"/>
@@ -834,6 +859,7 @@
       <c r="F14" s="6" t="inlineStr"/>
       <c r="G14" s="6" t="inlineStr"/>
       <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="6" t="inlineStr"/>
@@ -844,20 +870,21 @@
       <c r="F15" s="6" t="inlineStr"/>
       <c r="G15" s="6" t="inlineStr"/>
       <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H15"/>
+  <autoFilter ref="A1:I15"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation sqref="B3:B50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Área" error="Elige un área de la lista" promptTitle="Área" prompt="Área de la empresa" type="list">
+    <dataValidation sqref="B3:B50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Ventas,Marketing,Compras,Operaciones,Servicio,Administración"</formula1>
     </dataValidation>
     <dataValidation sqref="C3:C50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Tiempo completo,Medio tiempo,Por proyecto,Prácticas"</formula1>
     </dataValidation>
-    <dataValidation sqref="H3:H50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="¿Abierta?" prompt="Sí = se publica abierta" type="list">
+    <dataValidation sqref="H3:H50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -872,11 +899,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="88" customWidth="1" min="2" max="2"/>
+    <col width="92" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -898,7 +925,7 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
-          <t>Llenar una fila por vacante. Con eso se actualiza bolsa-trabajo.html en el sitio.</t>
+          <t>Llenar una fila por vacante. Con eso se actualiza la bolsa de trabajo en el sitio.</t>
         </is>
       </c>
     </row>
@@ -910,121 +937,121 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Solo lo de la hoja Vacantes: puesto, etiquetas, descripción corta y fechas.</t>
+          <t>Puesto, etiquetas, descripción corta, fechas y, si lo llenas, el link de OCC/externo.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Link OCC / externo</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Opcional. Pega la URL completa (https://...). Si está vacío, no se muestra botón externo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Qué NO hace falta</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Requisitos largos, sueldo, beneficios, CV, etc. Eso no se muestra en las tarjetas.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr"/>
-      <c r="B6" s="8" t="inlineStr"/>
-    </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr"/>
+      <c r="B7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Cómo llenar</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Ve a la hoja «Vacantes».</t>
-        </is>
-      </c>
+      <c r="B8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Borra o edita los ejemplos y agrega filas nuevas.</t>
+          <t>Ve a la hoja «Vacantes».</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Usa las listas desplegables (Área, Tipo, ¿Abierta?).</t>
+          <t>Borra o edita los ejemplos y agrega filas nuevas.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Fechas en formato AAAA-MM-DD (ej. 2026-07-29).</t>
+          <t>Usa las listas desplegables (Área, Tipo, ¿Abierta?).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Descripción: máximo 1–2 oraciones claras.</t>
+          <t>Fechas en formato AAAA-MM-DD (ej. 2026-07-29).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Si ya publicaron en OCC u otra bolsa, pega el link en la última columna.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Envía este archivo a quien publica la web.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr"/>
-      <c r="B14" s="8" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Campos obligatorios</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Puesto · Área · Tipo · Zona/detalle · Descripción · Publicación · Cierre · ¿Abierta?</t>
-        </is>
-      </c>
+      <c r="A15" s="8" t="inlineStr"/>
+      <c r="B15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
@@ -1034,7 +1061,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Se muestra en «Vacantes abiertas» (tarjeta grande) y en el catálogo.</t>
+          <t>Se muestra en «Vacantes abiertas» y en el catálogo.</t>
         </is>
       </c>
     </row>
@@ -1047,30 +1074,6 @@
       <c r="B17" s="8" t="inlineStr">
         <is>
           <t>Solo aparece en el catálogo como «Sin vacante activa».</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>Ejemplo de descripción buena</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>Asesoría y venta de soluciones AT&amp;T con respaldo YAAVS. Acompañas puntos de venta y cierras oportunidades en retail.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>Ejemplo malo (evitar)</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>Se requiere experiencia de 5 años, inglés avanzado, auto propio, disponibilidad de viajar, sueldo competitivo según perfil...</t>
         </is>
       </c>
     </row>

</xml_diff>